<commit_message>
I mean yeah pretty much working i guess
</commit_message>
<xml_diff>
--- a/centerline_data.xlsx
+++ b/centerline_data.xlsx
@@ -8,53 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ethanbeddard/Documents/CFD/LBMAttempt1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF2A763E-950D-514C-A883-E125CF8175E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF11EB35-C6BE-674C-9475-6F43E974FA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="860" windowWidth="36000" windowHeight="22520" xr2:uid="{E1544EC1-52FD-F64A-BA20-FDD20D7B928A}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="22500" xr2:uid="{E1544EC1-52FD-F64A-BA20-FDD20D7B928A}"/>
   </bookViews>
   <sheets>
     <sheet name="centerline_data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">centerline_data!$H$261</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">centerline_data!$H$6:$H$261</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">centerline_data!$I$6:$I$515</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">centerline_data!$H$6:$H$515</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">centerline_data!$I$6:$I$515</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">centerline_data!$H$261</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">centerline_data!$H$6:$H$261</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">centerline_data!$I$6:$I$261</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">centerline_data!$J$261</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">centerline_data!$O$6:$O$28</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">centerline_data!$P$6:$P$28</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">centerline_data!$H$6:$H$515</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">centerline_data!$I$6:$I$261</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">centerline_data!$I$6:$I$515</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">centerline_data!$H$6:$H$515</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">centerline_data!$I$5</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">centerline_data!$I$6:$I$515</definedName>
-    <definedName name="_xlchart.v1.36" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.37" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">centerline_data!$J$261</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">centerline_data!$K$6:$K$28</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">centerline_data!$L$6:$L$28</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">centerline_data!$O$6:$O$28</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">centerline_data!$P$6:$P$28</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">centerline_data!$H$6:$H$515</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -596,11 +556,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -8389,7 +8348,7 @@
       <c r="I141">
         <v>-2.3084005000000001E-2</v>
       </c>
-      <c r="J141" s="3">
+      <c r="J141" s="2">
         <v>7.4943000000000004E-5</v>
       </c>
     </row>

</xml_diff>